<commit_message>
invitation registry and customer service response
</commit_message>
<xml_diff>
--- a/docs/福利商城功能清单.xlsx
+++ b/docs/福利商城功能清单.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="447">
   <si>
     <t>福利商城平台层-功能清单</t>
   </si>
@@ -1762,11 +1762,6 @@
   </si>
   <si>
     <t>商城装修</t>
-  </si>
-  <si>
-    <t>1.商品销售数据、商城销售数据、分类销售数据
-2.供应链渠道数据、粉类销售数据
-3.卡券消费数据</t>
   </si>
   <si>
     <t>1.管理员设置（角色、权限、项目）
@@ -8528,14 +8523,14 @@
         <v>415</v>
       </c>
     </row>
-    <row r="20" ht="68" spans="1:6">
+    <row r="20" ht="51" spans="1:6">
       <c r="A20" s="13"/>
       <c r="B20" s="15" t="s">
         <v>431</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="12" t="s">
-        <v>441</v>
+        <v>432</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
@@ -8563,7 +8558,7 @@
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="19" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="10" t="s">
@@ -8572,14 +8567,14 @@
     </row>
     <row r="23" ht="76" customHeight="1" spans="1:6">
       <c r="A23" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="B23" s="22" t="s">
         <v>443</v>
-      </c>
-      <c r="B23" s="22" t="s">
-        <v>444</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="24" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E23" s="24"/>
       <c r="F23" s="24" t="s">
@@ -8588,12 +8583,12 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="25" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
       <c r="D24" s="25" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E24" s="25"/>
       <c r="F24" s="25" t="s">

</xml_diff>